<commit_message>
feat: INDEX + MATCH completo - Basico, Intermedio y Avanzado con busqueda entre hojas
</commit_message>
<xml_diff>
--- a/Atajos & Tecnicas.xlsx
+++ b/Atajos & Tecnicas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1d86eecf8daf4f0d/Documents/SQL Server Management Studio 22/Tienda-sqlserver/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2625AD05-6FBF-4852-93E5-1ABF9D00E33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{2625AD05-6FBF-4852-93E5-1ABF9D00E33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{039F1B1E-3171-43CA-AB7A-AE304DE27F59}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="12444" windowHeight="12240" activeTab="1" xr2:uid="{8AAA3391-6115-4541-868F-6CDF856BBE9F}"/>
   </bookViews>
@@ -1351,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37F40C96-7242-4A48-8F52-7EEFD866B4BA}">
-  <dimension ref="C3:K30"/>
+  <dimension ref="C3:K39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -1913,6 +1913,48 @@
         <v>Eduardo Castro Reyes</v>
       </c>
     </row>
+    <row r="33" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J33" t="str">
+        <f>_xlfn.CONCAT(C22, " ",D22, " ", E22)</f>
+        <v>Juan Ramirez Gonzales</v>
+      </c>
+    </row>
+    <row r="34" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J34" t="str">
+        <f t="shared" ref="J34:J39" si="2">_xlfn.CONCAT(C23, " ",D23, " ", E23)</f>
+        <v>Pedro Alvarez Alvarez</v>
+      </c>
+    </row>
+    <row r="35" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J35" t="str">
+        <f t="shared" si="2"/>
+        <v>Pamela Angular Benitez</v>
+      </c>
+    </row>
+    <row r="36" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J36" t="str">
+        <f t="shared" si="2"/>
+        <v>Julieta Castañeda Castro</v>
+      </c>
+    </row>
+    <row r="37" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J37" t="str">
+        <f t="shared" si="2"/>
+        <v>Ernesto Hernandez Hernandez</v>
+      </c>
+    </row>
+    <row r="38" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J38" t="str">
+        <f t="shared" si="2"/>
+        <v>Fernando Muñoz Cervantes</v>
+      </c>
+    </row>
+    <row r="39" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J39" t="str">
+        <f t="shared" si="2"/>
+        <v>Alicia Reyes Rivas</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="E4:F4"/>

</xml_diff>